<commit_message>
Final QA: update Item 41 category to Plaster
</commit_message>
<xml_diff>
--- a/output/passport_filled.xlsx
+++ b/output/passport_filled.xlsx
@@ -6148,7 +6148,7 @@
       </c>
       <c r="J47" s="8" t="inlineStr">
         <is>
-          <t>Flooring</t>
+          <t>Plaster</t>
         </is>
       </c>
       <c r="K47" s="8" t="inlineStr">
@@ -6180,9 +6180,13 @@
       <c r="U47" s="8" t="n"/>
       <c r="V47" s="8" t="n"/>
       <c r="W47" s="8" t="n"/>
-      <c r="X47" s="8" t="n"/>
+      <c r="X47" s="8" t="n">
+        <v>2000</v>
+      </c>
       <c r="Y47" s="8" t="n"/>
-      <c r="Z47" s="8" t="n"/>
+      <c r="Z47" s="8" t="n">
+        <v>0.18</v>
+      </c>
       <c r="AA47" s="8" t="inlineStr">
         <is>
           <t>DSR 1989</t>
@@ -6196,7 +6200,7 @@
       <c r="AC47" s="8" t="n"/>
       <c r="AD47" s="8" t="inlineStr">
         <is>
-          <t>Cement Skirting</t>
+          <t>Cement Plaster Skirting Render</t>
         </is>
       </c>
       <c r="AE47" s="8" t="n"/>
@@ -6224,7 +6228,7 @@
       </c>
       <c r="AX47" s="8" t="inlineStr">
         <is>
-          <t>Material-specific carbon factors excluded due to composite or specialized scope.</t>
+          <t>GWP: 0.180 kg CO2e/kg, Density: 2000 kg/m³ | Source: ICE Database v3.0 (Cement Mortar / Plaster).</t>
         </is>
       </c>
     </row>

</xml_diff>